<commit_message>
:herb: filter ASVs on prevalence + presence in groups with at least 2 samples
</commit_message>
<xml_diff>
--- a/data/derived_data/2_RarefyData/Dataset_1/ps_16S_filt_Dataset_1_tax_table.xlsx
+++ b/data/derived_data/2_RarefyData/Dataset_1/ps_16S_filt_Dataset_1_tax_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -38,40 +38,70 @@
     <t xml:space="preserve">Species</t>
   </si>
   <si>
-    <t xml:space="preserve">Cluster_1126</t>
+    <t xml:space="preserve">Cluster_10</t>
   </si>
   <si>
     <t xml:space="preserve">Bacteria</t>
   </si>
   <si>
+    <t xml:space="preserve">Bacillota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bacilli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lactobacillales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lactobacillaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fructilactobacillus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unknown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster_11</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pseudomonadota</t>
   </si>
   <si>
+    <t xml:space="preserve">Alphaproteobacteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acetobacterales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acetobacteraceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gluconobacter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster_113</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gammaproteobacteria</t>
   </si>
   <si>
     <t xml:space="preserve">Burkholderiales</t>
   </si>
   <si>
-    <t xml:space="preserve">Neisseriaceae</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Snodgrassella</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Snodgrassella alvi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_113</t>
-  </si>
-  <si>
     <t xml:space="preserve">Oxalobacteraceae</t>
   </si>
   <si>
     <t xml:space="preserve">Massilia</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown</t>
+    <t xml:space="preserve">Cluster_14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levilactobacillus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lactobacillus brevis</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_16</t>
@@ -83,24 +113,33 @@
     <t xml:space="preserve">Erwiniaceae</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gluconobacter wancherniae</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_20</t>
   </si>
   <si>
-    <t xml:space="preserve">Alphaproteobacteria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acetobacterales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acetobacteraceae</t>
-  </si>
-  <si>
     <t xml:space="preserve">Acetobacter</t>
   </si>
   <si>
     <t xml:space="preserve">Acetobacter thailandicus</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bacillales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planococcaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lysinibacillus</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_31</t>
   </si>
   <si>
@@ -113,58 +152,31 @@
     <t xml:space="preserve">Tatumella</t>
   </si>
   <si>
-    <t xml:space="preserve">Cluster_338</t>
+    <t xml:space="preserve">Cluster_5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster_53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bacillaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bacillus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster_6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gluconobacter cerinus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster_7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster_87</t>
   </si>
   <si>
     <t xml:space="preserve">Yersiniaceae</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serratia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serratia symbiotica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phaseolibacter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_53</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bacillota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bacilli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bacillales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bacillaceae</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bacillus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gluconobacter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gluconobacter cerinus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_87</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_9</t>
@@ -556,53 +568,53 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -611,102 +623,102 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H6" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
         <v>21</v>
       </c>
-      <c r="F7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" t="s">
-        <v>32</v>
-      </c>
       <c r="H7" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
@@ -718,68 +730,68 @@
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="F9" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H9" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G10" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="H10" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="F11" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="G11" t="s">
         <v>45</v>
       </c>
       <c r="H11" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -790,27 +802,27 @@
         <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H12" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B13" t="s">
         <v>9</v>
@@ -819,19 +831,19 @@
         <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="F13" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="G13" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="H13" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
@@ -842,48 +854,100 @@
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E14" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" t="s">
         <v>21</v>
       </c>
-      <c r="F14" t="s">
-        <v>34</v>
-      </c>
-      <c r="G14" t="s">
-        <v>19</v>
-      </c>
       <c r="H14" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D15" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G15" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="H15" t="s">
-        <v>28</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H17" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>